<commit_message>
Big boys Missing acc OL
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/ENSU.OL.xlsx
+++ b/data/obx_xlsx/ENSU.OL.xlsx
@@ -1056,7 +1056,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1137,6 +1137,9 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -7816,9 +7819,15 @@
       <c r="P28" s="15">
         <v>0.14</v>
       </c>
-      <c r="Q28" s="16"/>
-      <c r="R28" s="16"/>
-      <c r="S28" s="16"/>
+      <c r="Q28" s="27">
+        <v>0.0</v>
+      </c>
+      <c r="R28" s="27">
+        <v>0.0</v>
+      </c>
+      <c r="S28" s="27">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
@@ -8241,11 +8250,26 @@
       <c r="N39" s="15">
         <v>2.73</v>
       </c>
-      <c r="O39" s="15"/>
-      <c r="P39" s="15"/>
-      <c r="Q39" s="15"/>
-      <c r="R39" s="15"/>
-      <c r="S39" s="15"/>
+      <c r="O39" s="15">
+        <f t="shared" ref="O39:S39" si="1">O58</f>
+        <v>1.34</v>
+      </c>
+      <c r="P39" s="15">
+        <f t="shared" si="1"/>
+        <v>0.76</v>
+      </c>
+      <c r="Q39" s="15">
+        <f t="shared" si="1"/>
+        <v>0.17</v>
+      </c>
+      <c r="R39" s="15">
+        <f t="shared" si="1"/>
+        <v>0.74</v>
+      </c>
+      <c r="S39" s="15">
+        <f t="shared" si="1"/>
+        <v>0.39</v>
+      </c>
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
@@ -15393,1158 +15417,1158 @@
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="28" t="s">
         <v>280</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="28"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+      <c r="S20" s="29"/>
+      <c r="T20" s="29"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="30" t="s">
         <v>280</v>
       </c>
-      <c r="B21" s="30">
+      <c r="B21" s="31">
         <v>862.72</v>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="31">
         <v>456.05</v>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="31">
         <v>630.71</v>
       </c>
-      <c r="E21" s="30">
+      <c r="E21" s="31">
         <v>1381.12</v>
       </c>
-      <c r="F21" s="30">
+      <c r="F21" s="31">
         <v>726.96</v>
       </c>
-      <c r="G21" s="30">
+      <c r="G21" s="31">
         <v>299.29</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="31">
         <v>700.09</v>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="31">
         <v>2205.09</v>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="31">
         <v>2198.73</v>
       </c>
-      <c r="K21" s="30">
+      <c r="K21" s="31">
         <v>1969.52</v>
       </c>
-      <c r="L21" s="30">
+      <c r="L21" s="31">
         <v>2346.26</v>
       </c>
-      <c r="M21" s="30">
+      <c r="M21" s="31">
         <v>2528.48</v>
       </c>
-      <c r="N21" s="30">
+      <c r="N21" s="31">
         <v>649.99</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="31">
         <v>479.93</v>
       </c>
-      <c r="P21" s="30">
+      <c r="P21" s="31">
         <v>266.14</v>
       </c>
-      <c r="Q21" s="30">
+      <c r="Q21" s="31">
         <v>178.01</v>
       </c>
-      <c r="R21" s="31">
+      <c r="R21" s="32">
         <v>43.1</v>
       </c>
-      <c r="S21" s="30">
+      <c r="S21" s="31">
         <v>176.75</v>
       </c>
-      <c r="T21" s="30">
+      <c r="T21" s="31">
         <v>114.88</v>
       </c>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="30" t="s">
         <v>281</v>
       </c>
-      <c r="B22" s="30">
+      <c r="B22" s="31">
         <v>970.31</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="31">
         <v>780.5</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="31">
         <v>825.04</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="31">
         <v>1101.53</v>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="31">
         <v>1240.6</v>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="31">
         <v>1511.98</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="31">
         <v>1971.53</v>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="31">
         <v>2424.14</v>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="31">
         <v>2288.85</v>
       </c>
-      <c r="K22" s="30">
+      <c r="K22" s="31">
         <v>2034.49</v>
       </c>
-      <c r="L22" s="30">
+      <c r="L22" s="31">
         <v>1455.06</v>
       </c>
-      <c r="M22" s="30">
+      <c r="M22" s="31">
         <v>837.63</v>
       </c>
-      <c r="N22" s="30">
+      <c r="N22" s="31">
         <v>311.29</v>
       </c>
-      <c r="O22" s="30">
+      <c r="O22" s="31">
         <v>233.65</v>
       </c>
-      <c r="P22" s="30">
+      <c r="P22" s="31">
         <v>155.56</v>
       </c>
-      <c r="Q22" s="32"/>
-      <c r="R22" s="32"/>
-      <c r="S22" s="32"/>
-      <c r="T22" s="32"/>
+      <c r="Q22" s="33"/>
+      <c r="R22" s="33"/>
+      <c r="S22" s="33"/>
+      <c r="T22" s="33"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="28" t="s">
         <v>282</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="28"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
-      <c r="O23" s="28"/>
-      <c r="P23" s="28"/>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
-      <c r="T23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="29"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="29"/>
+      <c r="S23" s="29"/>
+      <c r="T23" s="29"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="30" t="s">
         <v>282</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="31">
         <v>757.23</v>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="31">
         <v>319.76</v>
       </c>
-      <c r="D24" s="30">
+      <c r="D24" s="31">
         <v>462.96</v>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="31">
         <v>1248.75</v>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="31">
         <v>551.91</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="31">
         <v>136.52</v>
       </c>
-      <c r="H24" s="30">
+      <c r="H24" s="31">
         <v>876.56</v>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="31">
         <v>2906.24</v>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="31">
         <v>2727.65</v>
       </c>
-      <c r="K24" s="30">
+      <c r="K24" s="31">
         <v>2110.42</v>
       </c>
-      <c r="L24" s="30">
+      <c r="L24" s="31">
         <v>2576.8</v>
       </c>
-      <c r="M24" s="30">
+      <c r="M24" s="31">
         <v>2794.92</v>
       </c>
-      <c r="N24" s="30">
+      <c r="N24" s="31">
         <v>682.84</v>
       </c>
-      <c r="O24" s="30">
+      <c r="O24" s="31">
         <v>487.27</v>
       </c>
-      <c r="P24" s="30">
+      <c r="P24" s="31">
         <v>284.2</v>
       </c>
-      <c r="Q24" s="30">
+      <c r="Q24" s="31">
         <v>187.85</v>
       </c>
-      <c r="R24" s="31">
+      <c r="R24" s="32">
         <v>52.39</v>
       </c>
-      <c r="S24" s="30">
+      <c r="S24" s="31">
         <v>196.24</v>
       </c>
-      <c r="T24" s="30">
+      <c r="T24" s="31">
         <v>114.88</v>
       </c>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="30" t="s">
         <v>283</v>
       </c>
-      <c r="B25" s="30">
+      <c r="B25" s="31">
         <v>799.16</v>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="31">
         <v>609.11</v>
       </c>
-      <c r="D25" s="30">
+      <c r="D25" s="31">
         <v>725.75</v>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="31">
         <v>1192.91</v>
       </c>
-      <c r="F25" s="30">
+      <c r="F25" s="31">
         <v>1460.45</v>
       </c>
-      <c r="G25" s="30">
+      <c r="G25" s="31">
         <v>1800.78</v>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="31">
         <v>2341.08</v>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="31">
         <v>2813.78</v>
       </c>
-      <c r="J25" s="30">
+      <c r="J25" s="31">
         <v>2561.54</v>
       </c>
-      <c r="K25" s="30">
+      <c r="K25" s="31">
         <v>2207.49</v>
       </c>
-      <c r="L25" s="30">
+      <c r="L25" s="31">
         <v>1582.09</v>
       </c>
-      <c r="M25" s="30">
+      <c r="M25" s="31">
         <v>905.39</v>
       </c>
-      <c r="N25" s="30">
+      <c r="N25" s="31">
         <v>326.06</v>
       </c>
-      <c r="O25" s="30">
+      <c r="O25" s="31">
         <v>246.74</v>
       </c>
-      <c r="P25" s="30">
+      <c r="P25" s="31">
         <v>166.88</v>
       </c>
-      <c r="Q25" s="32"/>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32"/>
-      <c r="T25" s="32"/>
+      <c r="Q25" s="33"/>
+      <c r="R25" s="33"/>
+      <c r="S25" s="33"/>
+      <c r="T25" s="33"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="28" t="s">
         <v>284</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
-      <c r="K26" s="28"/>
-      <c r="L26" s="28"/>
-      <c r="M26" s="28"/>
-      <c r="N26" s="28"/>
-      <c r="O26" s="28"/>
-      <c r="P26" s="28"/>
-      <c r="Q26" s="28"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
-      <c r="T26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
+      <c r="O26" s="29"/>
+      <c r="P26" s="29"/>
+      <c r="Q26" s="29"/>
+      <c r="R26" s="29"/>
+      <c r="S26" s="29"/>
+      <c r="T26" s="29"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="30" t="s">
         <v>285</v>
       </c>
-      <c r="B27" s="31">
+      <c r="B27" s="32">
         <v>1.08</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="32">
         <v>0.65</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="32">
         <v>9.15</v>
       </c>
-      <c r="E27" s="31">
+      <c r="E27" s="32">
         <v>31.07</v>
       </c>
-      <c r="F27" s="31">
+      <c r="F27" s="32">
         <v>24.33</v>
       </c>
-      <c r="G27" s="31">
+      <c r="G27" s="32">
         <v>49.4</v>
       </c>
-      <c r="H27" s="30">
+      <c r="H27" s="31">
         <v>317.2</v>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="31">
         <v>1051.69</v>
       </c>
-      <c r="J27" s="30">
+      <c r="J27" s="31">
         <v>1552.09</v>
       </c>
-      <c r="K27" s="30">
+      <c r="K27" s="31">
         <v>1611.46</v>
       </c>
-      <c r="L27" s="30">
+      <c r="L27" s="31">
         <v>2120.34</v>
       </c>
-      <c r="M27" s="30">
+      <c r="M27" s="31">
         <v>2518.96</v>
       </c>
-      <c r="N27" s="30">
+      <c r="N27" s="31">
         <v>818.45</v>
       </c>
-      <c r="O27" s="30">
+      <c r="O27" s="31">
         <v>678.51</v>
       </c>
-      <c r="P27" s="30">
+      <c r="P27" s="31">
         <v>432.55</v>
       </c>
-      <c r="Q27" s="30">
+      <c r="Q27" s="31">
         <v>547.05</v>
       </c>
-      <c r="R27" s="30">
+      <c r="R27" s="31">
         <v>209.09</v>
       </c>
-      <c r="S27" s="30">
+      <c r="S27" s="31">
         <v>836.35</v>
       </c>
-      <c r="T27" s="30">
+      <c r="T27" s="31">
         <v>585.45</v>
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="30" t="s">
         <v>286</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="32">
         <v>16.95</v>
       </c>
-      <c r="C28" s="31">
+      <c r="C28" s="32">
         <v>26.33</v>
       </c>
-      <c r="D28" s="31">
+      <c r="D28" s="32">
         <v>97.27</v>
       </c>
-      <c r="E28" s="30">
+      <c r="E28" s="31">
         <v>311.5</v>
       </c>
-      <c r="F28" s="30">
+      <c r="F28" s="31">
         <v>605.65</v>
       </c>
-      <c r="G28" s="30">
+      <c r="G28" s="31">
         <v>934.88</v>
       </c>
-      <c r="H28" s="30">
+      <c r="H28" s="31">
         <v>1400.56</v>
       </c>
-      <c r="I28" s="30">
+      <c r="I28" s="31">
         <v>1951.87</v>
       </c>
-      <c r="J28" s="30">
+      <c r="J28" s="31">
         <v>2086.93</v>
       </c>
-      <c r="K28" s="30">
+      <c r="K28" s="31">
         <v>2018.93</v>
       </c>
-      <c r="L28" s="30">
+      <c r="L28" s="31">
         <v>1545.15</v>
       </c>
-      <c r="M28" s="30">
+      <c r="M28" s="31">
         <v>1024.74</v>
       </c>
-      <c r="N28" s="30">
+      <c r="N28" s="31">
         <v>511.22</v>
       </c>
-      <c r="O28" s="30">
+      <c r="O28" s="31">
         <v>557.32</v>
       </c>
-      <c r="P28" s="30">
+      <c r="P28" s="31">
         <v>520.06</v>
       </c>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="32"/>
+      <c r="Q28" s="33"/>
+      <c r="R28" s="33"/>
+      <c r="S28" s="33"/>
+      <c r="T28" s="33"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="28" t="s">
         <v>287</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
-      <c r="T29" s="28"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="29"/>
+      <c r="M29" s="29"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="29"/>
+      <c r="P29" s="29"/>
+      <c r="Q29" s="29"/>
+      <c r="R29" s="29"/>
+      <c r="S29" s="29"/>
+      <c r="T29" s="29"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="30" t="s">
         <v>288</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="34">
         <v>-28.04</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="34">
         <v>-48.07</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <v>-46.04</v>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="34">
         <v>-17.57</v>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="34">
         <v>-59.7</v>
       </c>
-      <c r="G30" s="33">
+      <c r="G30" s="34">
         <v>-228.12</v>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="34">
         <v>-63.54</v>
       </c>
-      <c r="I30" s="33">
+      <c r="I30" s="34">
         <v>-30.62</v>
       </c>
-      <c r="J30" s="33">
+      <c r="J30" s="34">
         <v>-15.26</v>
       </c>
-      <c r="K30" s="33">
+      <c r="K30" s="34">
         <v>-13.62</v>
       </c>
-      <c r="L30" s="33">
+      <c r="L30" s="34">
         <v>-8.36</v>
       </c>
-      <c r="M30" s="33">
+      <c r="M30" s="34">
         <v>-2.79</v>
       </c>
-      <c r="N30" s="33">
+      <c r="N30" s="34">
         <v>-6.12</v>
       </c>
-      <c r="O30" s="33">
+      <c r="O30" s="34">
         <v>-7.57</v>
       </c>
-      <c r="P30" s="33">
+      <c r="P30" s="34">
         <v>-9.87</v>
       </c>
-      <c r="Q30" s="33">
+      <c r="Q30" s="34">
         <v>-10.79</v>
       </c>
-      <c r="R30" s="33">
+      <c r="R30" s="34">
         <v>-59.65</v>
       </c>
-      <c r="S30" s="33">
+      <c r="S30" s="34">
         <v>-12.49</v>
       </c>
-      <c r="T30" s="33">
+      <c r="T30" s="34">
         <v>-23.67</v>
       </c>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="30" t="s">
         <v>289</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="34">
         <v>-37.55</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="34">
         <v>-120.18</v>
       </c>
-      <c r="D31" s="33">
+      <c r="D31" s="34">
         <v>-78.38</v>
       </c>
-      <c r="E31" s="33">
+      <c r="E31" s="34">
         <v>-43.95</v>
       </c>
-      <c r="F31" s="33">
+      <c r="F31" s="34">
         <v>-29.61</v>
       </c>
-      <c r="G31" s="33">
+      <c r="G31" s="34">
         <v>-23.98</v>
       </c>
-      <c r="H31" s="33">
+      <c r="H31" s="34">
         <v>-17.09</v>
       </c>
-      <c r="I31" s="33">
+      <c r="I31" s="34">
         <v>-10.66</v>
       </c>
-      <c r="J31" s="33">
+      <c r="J31" s="34">
         <v>-7.99</v>
       </c>
-      <c r="K31" s="33">
+      <c r="K31" s="34">
         <v>-6.8</v>
       </c>
-      <c r="L31" s="33">
+      <c r="L31" s="34">
         <v>-5.82</v>
       </c>
-      <c r="M31" s="33">
+      <c r="M31" s="34">
         <v>-5.53</v>
       </c>
-      <c r="N31" s="33">
+      <c r="N31" s="34">
         <v>-11.55</v>
       </c>
-      <c r="O31" s="33">
+      <c r="O31" s="34">
         <v>-13.57</v>
       </c>
-      <c r="P31" s="33">
+      <c r="P31" s="34">
         <v>-17.22</v>
       </c>
-      <c r="Q31" s="34"/>
-      <c r="R31" s="34"/>
-      <c r="S31" s="34"/>
-      <c r="T31" s="34"/>
+      <c r="Q31" s="35"/>
+      <c r="R31" s="35"/>
+      <c r="S31" s="35"/>
+      <c r="T31" s="35"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="28" t="s">
         <v>290</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
-      <c r="T32" s="28"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="29"/>
+      <c r="P32" s="29"/>
+      <c r="Q32" s="29"/>
+      <c r="R32" s="29"/>
+      <c r="S32" s="29"/>
+      <c r="T32" s="29"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="30" t="s">
         <v>291</v>
       </c>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="31">
+      <c r="B33" s="33"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="33"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="33"/>
+      <c r="H33" s="32">
         <v>1.71</v>
       </c>
-      <c r="I33" s="31">
+      <c r="I33" s="32">
         <v>2.74</v>
       </c>
-      <c r="J33" s="31">
+      <c r="J33" s="32">
         <v>4.16</v>
       </c>
-      <c r="K33" s="31">
+      <c r="K33" s="32">
         <v>9.72</v>
       </c>
-      <c r="L33" s="31">
+      <c r="L33" s="32">
         <v>9.53</v>
       </c>
-      <c r="M33" s="31">
+      <c r="M33" s="32">
         <v>10.91</v>
       </c>
-      <c r="N33" s="31">
+      <c r="N33" s="32">
         <v>22.73</v>
       </c>
-      <c r="O33" s="30">
+      <c r="O33" s="31">
         <v>112.91</v>
       </c>
-      <c r="P33" s="31">
+      <c r="P33" s="32">
         <v>19.01</v>
       </c>
-      <c r="Q33" s="31">
+      <c r="Q33" s="32">
         <v>30.66</v>
       </c>
-      <c r="R33" s="31">
+      <c r="R33" s="32">
         <v>11.15</v>
       </c>
-      <c r="S33" s="31">
+      <c r="S33" s="32">
         <v>17.5</v>
       </c>
-      <c r="T33" s="31">
+      <c r="T33" s="32">
         <v>8.18</v>
       </c>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="29" t="s">
+      <c r="A34" s="30" t="s">
         <v>292</v>
       </c>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="31">
+      <c r="B34" s="33"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="32">
         <v>4.23</v>
       </c>
-      <c r="E34" s="31">
+      <c r="E34" s="32">
         <v>3.0</v>
       </c>
-      <c r="F34" s="31">
+      <c r="F34" s="32">
         <v>3.45</v>
       </c>
-      <c r="G34" s="31">
+      <c r="G34" s="32">
         <v>4.32</v>
       </c>
-      <c r="H34" s="31">
+      <c r="H34" s="32">
         <v>5.06</v>
       </c>
-      <c r="I34" s="31">
+      <c r="I34" s="32">
         <v>6.73</v>
       </c>
-      <c r="J34" s="31">
+      <c r="J34" s="32">
         <v>8.87</v>
       </c>
-      <c r="K34" s="31">
+      <c r="K34" s="32">
         <v>12.14</v>
       </c>
-      <c r="L34" s="31">
+      <c r="L34" s="32">
         <v>13.05</v>
       </c>
-      <c r="M34" s="31">
+      <c r="M34" s="32">
         <v>16.08</v>
       </c>
-      <c r="N34" s="31">
+      <c r="N34" s="32">
         <v>26.77</v>
       </c>
-      <c r="O34" s="31">
+      <c r="O34" s="32">
         <v>23.93</v>
       </c>
-      <c r="P34" s="31">
+      <c r="P34" s="32">
         <v>14.91</v>
       </c>
-      <c r="Q34" s="32"/>
-      <c r="R34" s="32"/>
-      <c r="S34" s="32"/>
-      <c r="T34" s="32"/>
+      <c r="Q34" s="33"/>
+      <c r="R34" s="33"/>
+      <c r="S34" s="33"/>
+      <c r="T34" s="33"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="28" t="s">
         <v>293</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="28"/>
-      <c r="L35" s="28"/>
-      <c r="M35" s="28"/>
-      <c r="N35" s="28"/>
-      <c r="O35" s="28"/>
-      <c r="P35" s="28"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
-      <c r="T35" s="28"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+      <c r="L35" s="29"/>
+      <c r="M35" s="29"/>
+      <c r="N35" s="29"/>
+      <c r="O35" s="29"/>
+      <c r="P35" s="29"/>
+      <c r="Q35" s="29"/>
+      <c r="R35" s="29"/>
+      <c r="S35" s="29"/>
+      <c r="T35" s="29"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="30" t="s">
         <v>294</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="31">
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="32">
         <v>1.78</v>
       </c>
-      <c r="I36" s="31">
+      <c r="I36" s="32">
         <v>2.78</v>
       </c>
-      <c r="J36" s="31">
+      <c r="J36" s="32">
         <v>4.32</v>
       </c>
-      <c r="K36" s="31">
+      <c r="K36" s="32">
         <v>10.87</v>
       </c>
-      <c r="L36" s="31">
+      <c r="L36" s="32">
         <v>10.18</v>
       </c>
-      <c r="M36" s="31">
+      <c r="M36" s="32">
         <v>10.91</v>
       </c>
-      <c r="N36" s="31">
+      <c r="N36" s="32">
         <v>22.73</v>
       </c>
-      <c r="O36" s="30">
+      <c r="O36" s="31">
         <v>112.9</v>
       </c>
-      <c r="P36" s="31">
+      <c r="P36" s="32">
         <v>19.02</v>
       </c>
-      <c r="Q36" s="31">
+      <c r="Q36" s="32">
         <v>30.66</v>
       </c>
-      <c r="R36" s="31">
+      <c r="R36" s="32">
         <v>11.16</v>
       </c>
-      <c r="S36" s="31">
+      <c r="S36" s="32">
         <v>16.82</v>
       </c>
-      <c r="T36" s="31">
+      <c r="T36" s="32">
         <v>8.28</v>
       </c>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="30" t="s">
         <v>295</v>
       </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="31">
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="32">
         <v>4.56</v>
       </c>
-      <c r="E37" s="31">
+      <c r="E37" s="32">
         <v>3.09</v>
       </c>
-      <c r="F37" s="31">
+      <c r="F37" s="32">
         <v>3.56</v>
       </c>
-      <c r="G37" s="31">
+      <c r="G37" s="32">
         <v>4.51</v>
       </c>
-      <c r="H37" s="31">
+      <c r="H37" s="32">
         <v>5.3</v>
       </c>
-      <c r="I37" s="31">
+      <c r="I37" s="32">
         <v>6.98</v>
       </c>
-      <c r="J37" s="31">
+      <c r="J37" s="32">
         <v>9.24</v>
       </c>
-      <c r="K37" s="31">
+      <c r="K37" s="32">
         <v>12.66</v>
       </c>
-      <c r="L37" s="31">
+      <c r="L37" s="32">
         <v>13.38</v>
       </c>
-      <c r="M37" s="31">
+      <c r="M37" s="32">
         <v>16.08</v>
       </c>
-      <c r="N37" s="31">
+      <c r="N37" s="32">
         <v>26.77</v>
       </c>
-      <c r="O37" s="31">
+      <c r="O37" s="32">
         <v>23.5</v>
       </c>
-      <c r="P37" s="31">
+      <c r="P37" s="32">
         <v>14.8</v>
       </c>
-      <c r="Q37" s="32"/>
-      <c r="R37" s="32"/>
-      <c r="S37" s="32"/>
-      <c r="T37" s="32"/>
+      <c r="Q37" s="33"/>
+      <c r="R37" s="33"/>
+      <c r="S37" s="33"/>
+      <c r="T37" s="33"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="28" t="s">
         <v>296</v>
       </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="28"/>
-      <c r="I38" s="28"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="28"/>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
-      <c r="O38" s="28"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
-      <c r="T38" s="28"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="29"/>
+      <c r="L38" s="29"/>
+      <c r="M38" s="29"/>
+      <c r="N38" s="29"/>
+      <c r="O38" s="29"/>
+      <c r="P38" s="29"/>
+      <c r="Q38" s="29"/>
+      <c r="R38" s="29"/>
+      <c r="S38" s="29"/>
+      <c r="T38" s="29"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="30" t="s">
         <v>297</v>
       </c>
-      <c r="B39" s="30">
+      <c r="B39" s="31">
         <v>939.93</v>
       </c>
-      <c r="C39" s="30">
+      <c r="C39" s="31">
         <v>229.47</v>
       </c>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="31">
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="32">
         <v>52.37</v>
       </c>
-      <c r="G39" s="31">
+      <c r="G39" s="32">
         <v>22.27</v>
       </c>
-      <c r="H39" s="31">
+      <c r="H39" s="32">
         <v>79.08</v>
       </c>
-      <c r="I39" s="31">
+      <c r="I39" s="32">
         <v>52.13</v>
       </c>
-      <c r="J39" s="31">
+      <c r="J39" s="32">
         <v>81.88</v>
       </c>
-      <c r="K39" s="31">
+      <c r="K39" s="32">
         <v>57.97</v>
       </c>
-      <c r="L39" s="31">
+      <c r="L39" s="32">
         <v>81.07</v>
       </c>
-      <c r="M39" s="30">
+      <c r="M39" s="31">
         <v>192.07</v>
       </c>
-      <c r="N39" s="30">
+      <c r="N39" s="31">
         <v>137.19</v>
       </c>
-      <c r="O39" s="30">
+      <c r="O39" s="31">
         <v>243.21</v>
       </c>
-      <c r="P39" s="30">
+      <c r="P39" s="31">
         <v>3483.7</v>
       </c>
-      <c r="Q39" s="31">
+      <c r="Q39" s="32">
         <v>40.61</v>
       </c>
-      <c r="R39" s="31">
+      <c r="R39" s="32">
         <v>22.24</v>
       </c>
-      <c r="S39" s="31">
+      <c r="S39" s="32">
         <v>64.52</v>
       </c>
-      <c r="T39" s="30">
+      <c r="T39" s="31">
         <v>219.36</v>
       </c>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="30" t="s">
         <v>298</v>
       </c>
-      <c r="B40" s="30">
+      <c r="B40" s="31">
         <v>136.72</v>
       </c>
-      <c r="C40" s="31">
+      <c r="C40" s="32">
         <v>42.29</v>
       </c>
-      <c r="D40" s="31">
+      <c r="D40" s="32">
         <v>64.37</v>
       </c>
-      <c r="E40" s="31">
+      <c r="E40" s="32">
         <v>54.76</v>
       </c>
-      <c r="F40" s="31">
+      <c r="F40" s="32">
         <v>65.08</v>
       </c>
-      <c r="G40" s="31">
+      <c r="G40" s="32">
         <v>62.54</v>
       </c>
-      <c r="H40" s="31">
+      <c r="H40" s="32">
         <v>68.92</v>
       </c>
-      <c r="I40" s="31">
+      <c r="I40" s="32">
         <v>88.35</v>
       </c>
-      <c r="J40" s="30">
+      <c r="J40" s="31">
         <v>100.06</v>
       </c>
-      <c r="K40" s="30">
+      <c r="K40" s="31">
         <v>110.37</v>
       </c>
-      <c r="L40" s="30">
+      <c r="L40" s="31">
         <v>143.15</v>
       </c>
-      <c r="M40" s="30">
+      <c r="M40" s="31">
         <v>139.66</v>
       </c>
-      <c r="N40" s="31">
+      <c r="N40" s="32">
         <v>87.69</v>
       </c>
-      <c r="O40" s="31">
+      <c r="O40" s="32">
         <v>71.16</v>
       </c>
-      <c r="P40" s="31">
+      <c r="P40" s="32">
         <v>68.57</v>
       </c>
-      <c r="Q40" s="32"/>
-      <c r="R40" s="32"/>
-      <c r="S40" s="32"/>
-      <c r="T40" s="32"/>
+      <c r="Q40" s="33"/>
+      <c r="R40" s="33"/>
+      <c r="S40" s="33"/>
+      <c r="T40" s="33"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="27" t="s">
+      <c r="A41" s="28" t="s">
         <v>299</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
-      <c r="K41" s="28"/>
-      <c r="L41" s="28"/>
-      <c r="M41" s="28"/>
-      <c r="N41" s="28"/>
-      <c r="O41" s="28"/>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="28"/>
-      <c r="S41" s="28"/>
-      <c r="T41" s="28"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="29"/>
+      <c r="K41" s="29"/>
+      <c r="L41" s="29"/>
+      <c r="M41" s="29"/>
+      <c r="N41" s="29"/>
+      <c r="O41" s="29"/>
+      <c r="P41" s="29"/>
+      <c r="Q41" s="29"/>
+      <c r="R41" s="29"/>
+      <c r="S41" s="29"/>
+      <c r="T41" s="29"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="30" t="s">
         <v>300</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="31">
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="32">
         <v>4.23</v>
       </c>
-      <c r="E42" s="31">
+      <c r="E42" s="32">
         <v>3.0</v>
       </c>
-      <c r="F42" s="31">
+      <c r="F42" s="32">
         <v>3.45</v>
       </c>
-      <c r="G42" s="31">
+      <c r="G42" s="32">
         <v>4.32</v>
       </c>
-      <c r="H42" s="31">
+      <c r="H42" s="32">
         <v>5.06</v>
       </c>
-      <c r="I42" s="31">
+      <c r="I42" s="32">
         <v>6.73</v>
       </c>
-      <c r="J42" s="31">
+      <c r="J42" s="32">
         <v>8.87</v>
       </c>
-      <c r="K42" s="31">
+      <c r="K42" s="32">
         <v>12.14</v>
       </c>
-      <c r="L42" s="31">
+      <c r="L42" s="32">
         <v>13.05</v>
       </c>
-      <c r="M42" s="31">
+      <c r="M42" s="32">
         <v>16.08</v>
       </c>
-      <c r="N42" s="31">
+      <c r="N42" s="32">
         <v>26.77</v>
       </c>
-      <c r="O42" s="31">
+      <c r="O42" s="32">
         <v>23.5</v>
       </c>
-      <c r="P42" s="31">
+      <c r="P42" s="32">
         <v>14.8</v>
       </c>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="32"/>
-      <c r="S42" s="32"/>
-      <c r="T42" s="32"/>
+      <c r="Q42" s="33"/>
+      <c r="R42" s="33"/>
+      <c r="S42" s="33"/>
+      <c r="T42" s="33"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="28" t="s">
         <v>301</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28"/>
-      <c r="M43" s="28"/>
-      <c r="N43" s="28"/>
-      <c r="O43" s="28"/>
-      <c r="P43" s="28"/>
-      <c r="Q43" s="28"/>
-      <c r="R43" s="28"/>
-      <c r="S43" s="28"/>
-      <c r="T43" s="28"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+      <c r="L43" s="29"/>
+      <c r="M43" s="29"/>
+      <c r="N43" s="29"/>
+      <c r="O43" s="29"/>
+      <c r="P43" s="29"/>
+      <c r="Q43" s="29"/>
+      <c r="R43" s="29"/>
+      <c r="S43" s="29"/>
+      <c r="T43" s="29"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="29" t="s">
+      <c r="A44" s="30" t="s">
         <v>302</v>
       </c>
-      <c r="B44" s="30">
+      <c r="B44" s="31">
         <v>1244.36</v>
       </c>
-      <c r="C44" s="30">
+      <c r="C44" s="31">
         <v>326.06</v>
       </c>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="30">
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="31">
         <v>172.25</v>
       </c>
-      <c r="G44" s="31">
+      <c r="G44" s="32">
         <v>48.64</v>
       </c>
-      <c r="H44" s="31">
+      <c r="H44" s="32">
         <v>62.92</v>
       </c>
-      <c r="I44" s="31">
+      <c r="I44" s="32">
         <v>53.52</v>
       </c>
-      <c r="J44" s="31">
+      <c r="J44" s="32">
         <v>74.35</v>
       </c>
-      <c r="K44" s="31">
+      <c r="K44" s="32">
         <v>55.63</v>
       </c>
-      <c r="L44" s="31">
+      <c r="L44" s="32">
         <v>78.72</v>
       </c>
-      <c r="M44" s="30">
+      <c r="M44" s="31">
         <v>212.23</v>
       </c>
-      <c r="N44" s="30">
+      <c r="N44" s="31">
         <v>139.43</v>
       </c>
-      <c r="O44" s="30">
+      <c r="O44" s="31">
         <v>255.39</v>
       </c>
-      <c r="P44" s="30">
+      <c r="P44" s="31">
         <v>4382.36</v>
       </c>
-      <c r="Q44" s="31">
+      <c r="Q44" s="32">
         <v>43.33</v>
       </c>
-      <c r="R44" s="31">
+      <c r="R44" s="32">
         <v>17.51</v>
       </c>
-      <c r="S44" s="31">
+      <c r="S44" s="32">
         <v>60.74</v>
       </c>
-      <c r="T44" s="30">
+      <c r="T44" s="31">
         <v>212.83</v>
       </c>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="29" t="s">
+      <c r="A45" s="30" t="s">
         <v>303</v>
       </c>
-      <c r="B45" s="30">
+      <c r="B45" s="31">
         <v>617.74</v>
       </c>
-      <c r="C45" s="30">
+      <c r="C45" s="31">
         <v>289.29</v>
       </c>
-      <c r="D45" s="30">
+      <c r="D45" s="31">
         <v>169.73</v>
       </c>
-      <c r="E45" s="31">
+      <c r="E45" s="32">
         <v>83.37</v>
       </c>
-      <c r="F45" s="31">
+      <c r="F45" s="32">
         <v>66.19</v>
       </c>
-      <c r="G45" s="31">
+      <c r="G45" s="32">
         <v>59.65</v>
       </c>
-      <c r="H45" s="31">
+      <c r="H45" s="32">
         <v>64.37</v>
       </c>
-      <c r="I45" s="31">
+      <c r="I45" s="32">
         <v>80.26</v>
       </c>
-      <c r="J45" s="31">
+      <c r="J45" s="32">
         <v>93.18</v>
       </c>
-      <c r="K45" s="30">
+      <c r="K45" s="31">
         <v>103.58</v>
       </c>
-      <c r="L45" s="30">
+      <c r="L45" s="31">
         <v>136.83</v>
       </c>
-      <c r="M45" s="30">
+      <c r="M45" s="31">
         <v>179.98</v>
       </c>
-      <c r="N45" s="30">
+      <c r="N45" s="31">
         <v>125.67</v>
       </c>
-      <c r="O45" s="30">
+      <c r="O45" s="31">
         <v>101.6</v>
       </c>
-      <c r="P45" s="31">
+      <c r="P45" s="32">
         <v>78.77</v>
       </c>
-      <c r="Q45" s="32"/>
-      <c r="R45" s="32"/>
-      <c r="S45" s="32"/>
-      <c r="T45" s="32"/>
+      <c r="Q45" s="33"/>
+      <c r="R45" s="33"/>
+      <c r="S45" s="33"/>
+      <c r="T45" s="33"/>
     </row>
     <row r="46" ht="15.75" customHeight="1"/>
     <row r="47" ht="15.75" customHeight="1"/>

</xml_diff>